<commit_message>
Update Feature_Story.xlsx with latest changes
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/Feature_Story.xlsx
+++ b/backlog/Feature_Story.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Documents\Ruchi_Office_Important\watch-datapipeline\backlog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA228170-1022-4382-B4AF-8DC23B5C67F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAC0862A-9368-47D1-99B1-808F22A0913C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10320" xr2:uid="{4CD1A7F7-4D43-438E-AADC-95F9EACC7B8E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="464">
   <si>
     <t>Feature</t>
   </si>
@@ -805,6 +805,627 @@
   </si>
   <si>
     <t>P0,Governance,Standards,Control</t>
+  </si>
+  <si>
+    <t>P1 Collector</t>
+  </si>
+  <si>
+    <t>Collector Architecture</t>
+  </si>
+  <si>
+    <t>P1-1A</t>
+  </si>
+  <si>
+    <t>Define Collector Capability Model Supporting ADOT and Custom Collector Implementations</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want a collector capability model so that both ADOT and custom collectors can be supported in a pluggable manner</t>
+  </si>
+  <si>
+    <t>Define capabilities, abstraction layer, pluggability model</t>
+  </si>
+  <si>
+    <t>collector-capability-model.md</t>
+  </si>
+  <si>
+    <t>Capability model supports both implementations</t>
+  </si>
+  <si>
+    <t>Simulate switching collectors via config</t>
+  </si>
+  <si>
+    <t>P1,Collector,OTEL,ADOT,CustomCollector,Pluggability</t>
+  </si>
+  <si>
+    <t>P1-1B</t>
+  </si>
+  <si>
+    <t>Define Collector Configuration Model for Implementation Selection</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want a configuration model so that collector implementation can be selected dynamically</t>
+  </si>
+  <si>
+    <t>Define config-driven mechanism to switch between ADOT and custom collector without code changes</t>
+  </si>
+  <si>
+    <t>Define config schema and selection logic</t>
+  </si>
+  <si>
+    <t>collector-config-schema.yaml</t>
+  </si>
+  <si>
+    <t>Config enables switching implementations</t>
+  </si>
+  <si>
+    <t>Validate config-based switching</t>
+  </si>
+  <si>
+    <t>P1,Collector,Config,Pluggability</t>
+  </si>
+  <si>
+    <t>Ingestion &amp; API Gateway</t>
+  </si>
+  <si>
+    <t>P1-2A</t>
+  </si>
+  <si>
+    <t>Define API Gateway as Standard Ingestion Aperture for Telemetry</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want API Gateway as ingestion layer so that all telemetry flows through a controlled entry point</t>
+  </si>
+  <si>
+    <t>Define API Gateway as mandatory ingestion layer ensuring decoupling and governance</t>
+  </si>
+  <si>
+    <t>Define ingestion architecture and flow</t>
+  </si>
+  <si>
+    <t>ingestion-architecture.md</t>
+  </si>
+  <si>
+    <t>All ingestion routed via gateway</t>
+  </si>
+  <si>
+    <t>Validate ingestion flow</t>
+  </si>
+  <si>
+    <t>P1,API,Gateway,Ingestion,Aperture</t>
+  </si>
+  <si>
+    <t>P1-2B</t>
+  </si>
+  <si>
+    <t>Implement Terraform Modules for API Gateway Provisioning</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want Terraform-based API Gateway setup so that environments can be provisioned consistently</t>
+  </si>
+  <si>
+    <t>Define Terraform modules for API Gateway provisioning integrated with platform infra</t>
+  </si>
+  <si>
+    <t>Define Terraform modules and configs</t>
+  </si>
+  <si>
+    <t>Terraform scripts for API Gateway</t>
+  </si>
+  <si>
+    <t>Gateway deployable via Terraform</t>
+  </si>
+  <si>
+    <t>Deploy in test environment</t>
+  </si>
+  <si>
+    <t>P1,Terraform,API,Infra</t>
+  </si>
+  <si>
+    <t>P1-2C</t>
+  </si>
+  <si>
+    <t>Define API Gateway Routing and Throttling Rules for Telemetry Ingestion</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want routing and throttling rules so that ingestion is scalable and controlled</t>
+  </si>
+  <si>
+    <t>Define routing rules, rate limits, and throttling for telemetry ingestion</t>
+  </si>
+  <si>
+    <t>Define routing policies and rate limits</t>
+  </si>
+  <si>
+    <t>API gateway configuration</t>
+  </si>
+  <si>
+    <t>Rules enforce ingestion control</t>
+  </si>
+  <si>
+    <t>Validate with load simulation</t>
+  </si>
+  <si>
+    <t>P1,API,Scaling,Throttling</t>
+  </si>
+  <si>
+    <t>Collector Implementation</t>
+  </si>
+  <si>
+    <t>P1-3A</t>
+  </si>
+  <si>
+    <t>Setup ADOT Collector with Standard Configuration</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want ADOT collector setup so that standard telemetry ingestion is supported</t>
+  </si>
+  <si>
+    <t>Configure ADOT collector with OTEL pipelines aligned to contracts</t>
+  </si>
+  <si>
+    <t>Define pipelines and exporters</t>
+  </si>
+  <si>
+    <t>ADOT config files</t>
+  </si>
+  <si>
+    <t>ADOT collector operational</t>
+  </si>
+  <si>
+    <t>Validate ingestion pipeline</t>
+  </si>
+  <si>
+    <t>P1,ADOT,OTEL,Collector</t>
+  </si>
+  <si>
+    <t>P1-3B</t>
+  </si>
+  <si>
+    <t>Develop Custom Collector for Advanced Processing (PII Redaction, Enrichment)</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want custom collector so that advanced capabilities like PII redaction are supported</t>
+  </si>
+  <si>
+    <t>Implement custom collector supporting transformation, redaction, enrichment</t>
+  </si>
+  <si>
+    <t>Define processing pipeline and logic</t>
+  </si>
+  <si>
+    <t>Custom collector implementation</t>
+  </si>
+  <si>
+    <t>PII redaction and enrichment working</t>
+  </si>
+  <si>
+    <t>Validate with sample data</t>
+  </si>
+  <si>
+    <t>P1,CustomCollector,PII,Processing</t>
+  </si>
+  <si>
+    <t>P1-3C</t>
+  </si>
+  <si>
+    <t>Define Processing Pipeline for Telemetry Transformation and Routing</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want processing pipeline so that telemetry can be transformed and routed appropriately</t>
+  </si>
+  <si>
+    <t>Define processing stages for enrichment, filtering, routing</t>
+  </si>
+  <si>
+    <t>Processing pipeline definition</t>
+  </si>
+  <si>
+    <t>Pipeline supports transformation</t>
+  </si>
+  <si>
+    <t>Validate pipeline outputs</t>
+  </si>
+  <si>
+    <t>P1,Processing,Pipeline</t>
+  </si>
+  <si>
+    <t>Contracts &amp; Integration</t>
+  </si>
+  <si>
+    <t>P1-4A</t>
+  </si>
+  <si>
+    <t>Integrate Telemetry Contract Enforcement in Collector Pipelines</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want contract enforcement so that all telemetry complies with platform standards</t>
+  </si>
+  <si>
+    <t>Ensure collector validates telemetry against defined contracts before processing</t>
+  </si>
+  <si>
+    <t>Integrate validation logic</t>
+  </si>
+  <si>
+    <t>Contract validation module</t>
+  </si>
+  <si>
+    <t>Invalid telemetry rejected</t>
+  </si>
+  <si>
+    <t>Test invalid payload</t>
+  </si>
+  <si>
+    <t>P1,Contracts,Validation</t>
+  </si>
+  <si>
+    <t>P1-4B</t>
+  </si>
+  <si>
+    <t>Implement Trace Propagation Across Collector Pipelines</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want trace propagation so that end-to-end observability is maintained</t>
+  </si>
+  <si>
+    <t>Ensure trace_id propagation across ingestion, processing, and export</t>
+  </si>
+  <si>
+    <t>Define propagation mechanism</t>
+  </si>
+  <si>
+    <t>Trace propagation implementation</t>
+  </si>
+  <si>
+    <t>Trace continuity maintained</t>
+  </si>
+  <si>
+    <t>Validate trace flow</t>
+  </si>
+  <si>
+    <t>P1,Tracing,OTEL</t>
+  </si>
+  <si>
+    <t>Infrastructure</t>
+  </si>
+  <si>
+    <t>P1-5A</t>
+  </si>
+  <si>
+    <t>Define Terraform Modules for Collector Deployment</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want Terraform modules so that collector can be deployed consistently</t>
+  </si>
+  <si>
+    <t>Define reusable Terraform modules for collector infra</t>
+  </si>
+  <si>
+    <t>Define infra modules</t>
+  </si>
+  <si>
+    <t>Terraform scripts</t>
+  </si>
+  <si>
+    <t>Collector deployable via Terraform</t>
+  </si>
+  <si>
+    <t>Deploy in test env</t>
+  </si>
+  <si>
+    <t>P1,Terraform,Infra</t>
+  </si>
+  <si>
+    <t>P1-5B</t>
+  </si>
+  <si>
+    <t>Enable Dual Deployment Strategy (Embedded and Portable)</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want dual deployment so that both platform-managed and user-managed setups are supported</t>
+  </si>
+  <si>
+    <t>Define deployment strategies for embedded and portable setups</t>
+  </si>
+  <si>
+    <t>Define deployment modes</t>
+  </si>
+  <si>
+    <t>Deployment strategy doc</t>
+  </si>
+  <si>
+    <t>Both modes supported</t>
+  </si>
+  <si>
+    <t>Validate both deployments</t>
+  </si>
+  <si>
+    <t>P1,Deployment,Packaging</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>P1-6A</t>
+  </si>
+  <si>
+    <t>Implement PII Detection and Redaction in Collector</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want PII redaction so that sensitive data is not exposed</t>
+  </si>
+  <si>
+    <t>Implement PII detection and masking in custom collector</t>
+  </si>
+  <si>
+    <t>Define detection and masking rules</t>
+  </si>
+  <si>
+    <t>PII processing module</t>
+  </si>
+  <si>
+    <t>PII properly redacted</t>
+  </si>
+  <si>
+    <t>P1,Security,PII</t>
+  </si>
+  <si>
+    <t>P1-6B</t>
+  </si>
+  <si>
+    <t>Secure Collector Endpoints and Ingestion Interfaces</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want secure endpoints so that ingestion is protected</t>
+  </si>
+  <si>
+    <t>Implement authentication and secure communication for collector endpoints</t>
+  </si>
+  <si>
+    <t>Define auth and encryption</t>
+  </si>
+  <si>
+    <t>Security configuration</t>
+  </si>
+  <si>
+    <t>Endpoints secured</t>
+  </si>
+  <si>
+    <t>Validate with auth tests</t>
+  </si>
+  <si>
+    <t>P1,Security,API</t>
+  </si>
+  <si>
+    <t>Define capability model covering ingestion, processing, transformation, routing, export supporting ADOT and custom collectors via configuration</t>
+  </si>
+  <si>
+    <t>Scaling &amp; Performance</t>
+  </si>
+  <si>
+    <t>P1-7A</t>
+  </si>
+  <si>
+    <t>Define Collector Horizontal Scaling Model for High-Volume Telemetry</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want a defined scaling model so that collector can handle varying telemetry loads without degradation</t>
+  </si>
+  <si>
+    <t>Define horizontal scaling approach including stateless design, load distribution, and scaling triggers aligned with cloud-native patterns</t>
+  </si>
+  <si>
+    <t>Define scaling architecture, stateless requirements, scaling triggers</t>
+  </si>
+  <si>
+    <t>scaling-model.md</t>
+  </si>
+  <si>
+    <t>Scaling model supports high throughput and horizontal scaling</t>
+  </si>
+  <si>
+    <t>Simulate load and validate scaling behavior</t>
+  </si>
+  <si>
+    <t>P1,Scaling,Performance,Architecture</t>
+  </si>
+  <si>
+    <t>P1-7B</t>
+  </si>
+  <si>
+    <t>Define Auto-Scaling Policies and Thresholds for Collector Infrastructure</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want auto-scaling policies so that collector dynamically adapts to workload</t>
+  </si>
+  <si>
+    <t>Define CPU, memory, throughput-based scaling thresholds and policies using Terraform/cloud configs</t>
+  </si>
+  <si>
+    <t>Define thresholds, policies, scaling rules</t>
+  </si>
+  <si>
+    <t>autoscaling-config.yaml</t>
+  </si>
+  <si>
+    <t>Auto-scaling triggers correctly based on load</t>
+  </si>
+  <si>
+    <t>Validate scaling under simulated load</t>
+  </si>
+  <si>
+    <t>P1,Scaling,Infra,Automation</t>
+  </si>
+  <si>
+    <t>Export &amp; Integration</t>
+  </si>
+  <si>
+    <t>P1-7C</t>
+  </si>
+  <si>
+    <t>Define Standard Export Contracts for Telemetry Delivery to Downstream Systems</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want export contracts so that telemetry is delivered consistently to downstream systems</t>
+  </si>
+  <si>
+    <t>Define contract for exporting logs, metrics, and traces ensuring compatibility with observability backends</t>
+  </si>
+  <si>
+    <t>Define export schema, formats, endpoints</t>
+  </si>
+  <si>
+    <t>export-contract.yaml</t>
+  </si>
+  <si>
+    <t>Export conforms to defined contract</t>
+  </si>
+  <si>
+    <t>Validate data in downstream system</t>
+  </si>
+  <si>
+    <t>P1,Export,Contracts,Integration</t>
+  </si>
+  <si>
+    <t>P1-7D</t>
+  </si>
+  <si>
+    <t>Implement Config-Driven Multi-Destination Telemetry Routing</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want configurable routing so that telemetry can be sent to multiple systems without code changes</t>
+  </si>
+  <si>
+    <t>Enable routing rules to direct telemetry to multiple destinations based on config and metadata</t>
+  </si>
+  <si>
+    <t>Define routing rules and config model</t>
+  </si>
+  <si>
+    <t>routing-config.yaml</t>
+  </si>
+  <si>
+    <t>Telemetry routed to multiple destinations correctly</t>
+  </si>
+  <si>
+    <t>Validate routing across endpoints</t>
+  </si>
+  <si>
+    <t>P1,Routing,Export,Config</t>
+  </si>
+  <si>
+    <t>Observability of Collector</t>
+  </si>
+  <si>
+    <t>P1-8A</t>
+  </si>
+  <si>
+    <t>Enable Self-Observability for Collector Components</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want collector to emit its own telemetry so that its health and behavior are observable</t>
+  </si>
+  <si>
+    <t>Instrument collector to emit metrics, logs, and traces aligned with telemetry contracts</t>
+  </si>
+  <si>
+    <t>Define self-observability signals</t>
+  </si>
+  <si>
+    <t>collector-observability-config</t>
+  </si>
+  <si>
+    <t>Collector emits internal telemetry</t>
+  </si>
+  <si>
+    <t>Validate collector metrics and traces</t>
+  </si>
+  <si>
+    <t>P1,Observability,Monitoring,Collector</t>
+  </si>
+  <si>
+    <t>P1-8B</t>
+  </si>
+  <si>
+    <t>Define Standard Health and Performance Metrics for Collector Monitoring</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want standardized metrics so that collector health can be monitored consistently</t>
+  </si>
+  <si>
+    <t>Define metrics like latency, throughput, error rate, and queue depth for monitoring</t>
+  </si>
+  <si>
+    <t>Define metric definitions and thresholds</t>
+  </si>
+  <si>
+    <t>health-metrics-definition.md</t>
+  </si>
+  <si>
+    <t>Metrics available and consistent</t>
+  </si>
+  <si>
+    <t>Validate metrics in monitoring system</t>
+  </si>
+  <si>
+    <t>P1,Monitoring,Health,Metrics</t>
+  </si>
+  <si>
+    <t>Resilience</t>
+  </si>
+  <si>
+    <t>P1-9A</t>
+  </si>
+  <si>
+    <t>Define Retry and Error Handling Strategy for Collector Pipelines</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want retry strategy so that transient failures do not cause data loss</t>
+  </si>
+  <si>
+    <t>Define retry logic, exponential backoff, and failure handling patterns for ingestion and processing</t>
+  </si>
+  <si>
+    <t>Define retry policies and error handling rules</t>
+  </si>
+  <si>
+    <t>retry-strategy.md</t>
+  </si>
+  <si>
+    <t>Retry mechanism handles transient failures</t>
+  </si>
+  <si>
+    <t>Simulate failure scenarios</t>
+  </si>
+  <si>
+    <t>P1,Resilience,Retry,ErrorHandling</t>
+  </si>
+  <si>
+    <t>P1-9B</t>
+  </si>
+  <si>
+    <t>Implement Buffering and Backpressure Handling Mechanisms</t>
+  </si>
+  <si>
+    <t>As a Data Engineering team, I want buffering so that burst traffic is handled without data loss or overload</t>
+  </si>
+  <si>
+    <t>Define buffering strategies, queueing mechanisms, and backpressure handling aligned with scaling model</t>
+  </si>
+  <si>
+    <t>Define buffering and queue strategies</t>
+  </si>
+  <si>
+    <t>buffering-config.yaml</t>
+  </si>
+  <si>
+    <t>No data loss under burst load</t>
+  </si>
+  <si>
+    <t>Load test with burst traffic</t>
+  </si>
+  <si>
+    <t>P1,Resilience,Buffering,Scaling</t>
   </si>
 </sst>
 </file>
@@ -855,7 +1476,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -863,6 +1484,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1177,19 +1799,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3594F0E7-7C10-4023-9C47-66514D348C6C}">
-  <dimension ref="A1:L28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L50"/>
+  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="9.140625" customWidth="1"/>
-    <col min="4" max="4" width="32.140625" customWidth="1"/>
-    <col min="5" max="5" width="40.7109375" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" customWidth="1"/>
-    <col min="8" max="10" width="9.140625" customWidth="1"/>
-    <col min="12" max="12" width="9.140625" customWidth="1"/>
+    <col min="1" max="2" width="9.140625" style="3"/>
+    <col min="3" max="3" width="9.140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="32.140625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="40.7109375" style="3" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" style="3" customWidth="1"/>
+    <col min="8" max="10" width="9.140625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" style="3"/>
+    <col min="12" max="12" width="9.140625" style="3" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1227,7 +1852,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="78.75" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -1265,7 +1890,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="56.25" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1303,7 +1928,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="45" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -1341,7 +1966,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="45" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -1379,7 +2004,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="45" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -1417,7 +2042,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="45" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -1455,7 +2080,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="45" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -1493,7 +2118,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -1531,7 +2156,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -1569,7 +2194,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -1607,7 +2232,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -1645,7 +2270,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="45" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
@@ -1683,7 +2308,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
@@ -1721,7 +2346,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="45" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>10</v>
       </c>
@@ -1759,7 +2384,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>10</v>
       </c>
@@ -1797,7 +2422,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>10</v>
       </c>
@@ -1835,7 +2460,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>10</v>
       </c>
@@ -1873,7 +2498,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" ht="45" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>10</v>
       </c>
@@ -1911,7 +2536,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>10</v>
       </c>
@@ -1949,7 +2574,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>10</v>
       </c>
@@ -1987,7 +2612,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="33.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>10</v>
       </c>
@@ -2025,7 +2650,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="101.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" ht="101.25" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>10</v>
       </c>
@@ -2063,7 +2688,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" ht="90" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>10</v>
       </c>
@@ -2101,7 +2726,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" ht="78.75" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>10</v>
       </c>
@@ -2139,7 +2764,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="67.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" ht="67.5" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>10</v>
       </c>
@@ -2177,7 +2802,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" ht="56.25" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>10</v>
       </c>
@@ -2215,7 +2840,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" ht="78.75" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>10</v>
       </c>
@@ -2251,6 +2876,842 @@
       </c>
       <c r="L28" s="2" t="s">
         <v>256</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" ht="101.25" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="K29" s="2">
+        <v>1</v>
+      </c>
+      <c r="L29" s="2" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="67.5" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="K30" s="2">
+        <v>1</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="56.25" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="K31" s="2">
+        <v>1</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="67.5" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="K32" s="2">
+        <v>1</v>
+      </c>
+      <c r="L32" s="2" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="45" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="K33" s="2">
+        <v>1</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" ht="45" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="K34" s="2">
+        <v>1</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="56.25" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="K35" s="2">
+        <v>1</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" ht="45" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="K36" s="2">
+        <v>1</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="56.25" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K37" s="2">
+        <v>1</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="56.25" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="K38" s="2">
+        <v>1</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" ht="45" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="K39" s="2">
+        <v>1</v>
+      </c>
+      <c r="L39" s="2" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" ht="45" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="K40" s="2">
+        <v>1</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" ht="45" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="K41" s="2">
+        <v>1</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" ht="56.25" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="K42" s="2">
+        <v>1</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="90" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="K43" s="2">
+        <v>1</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" ht="78.75" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="K44" s="2">
+        <v>1</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" ht="78.75" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="K45" s="2">
+        <v>1</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" ht="67.5" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="K46" s="2">
+        <v>1</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" ht="56.25" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="K47" s="2">
+        <v>1</v>
+      </c>
+      <c r="L47" s="2" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" ht="56.25" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="K48" s="2">
+        <v>1</v>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" ht="67.5" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="K49" s="2">
+        <v>1</v>
+      </c>
+      <c r="L49" s="2" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" ht="67.5" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="K50" s="2">
+        <v>1</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>463</v>
       </c>
     </row>
   </sheetData>

</xml_diff>